<commit_message>
feat: the certificate URL column was removed, as it is not used for now
</commit_message>
<xml_diff>
--- a/src/templates/formato_certificado_estandar.xlsx
+++ b/src/templates/formato_certificado_estandar.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://servimeters-my.sharepoint.com/personal/duvan_sanabria_servimeters_com/Documents/Documentos/Software/consulta_certificados/src/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\duvan.sanabria\OneDrive - Servimeters\Documentos\Software\consulta_certificados\src\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{877F5B5F-2FCD-42C2-930D-0073A15E86A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B8B7887-0340-4E15-8C22-6DCECE27BBE1}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B2F7DA1-FD0C-42C2-8FD1-9748DCEA46F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{627C57AE-B618-423A-8333-07391A41D1B5}"/>
+    <workbookView xWindow="35475" yWindow="1455" windowWidth="21600" windowHeight="11295" xr2:uid="{627C57AE-B618-423A-8333-07391A41D1B5}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="133">
   <si>
     <t>NOMBRE</t>
   </si>
@@ -44,22 +44,397 @@
     <t xml:space="preserve">CAPACITACION </t>
   </si>
   <si>
-    <t>URL</t>
+    <t>Pais</t>
+  </si>
+  <si>
+    <t>N° CERTIFICADO</t>
+  </si>
+  <si>
+    <t>#2AB0AMGGPN2@M0X3</t>
+  </si>
+  <si>
+    <t>ALBA AIDEE AGUILAR ABREGO</t>
   </si>
   <si>
     <t>AUDITOR INTERNO DE SISTEMAS DE GESTIÓN DE LA CALIDAD SEGÚN LA NORMA ISO 9001:2015</t>
   </si>
   <si>
-    <t>https://servimeters-my.sharepoint.com/:x:/r/personal/duvan_sanabria_servimeters_com/_layouts/15/Doc.aspx?sourcedoc=%7B9D631C9C-C83D-4260-8520-0BA5934135E4%7D&amp;file=Prog%20en%20Sitio-RICARDO.xlsx&amp;action=default&amp;mobileredirect=true&amp;DefaultItemOpen=1</t>
-  </si>
-  <si>
-    <t>Pais</t>
-  </si>
-  <si>
-    <t>Colombia</t>
-  </si>
-  <si>
-    <t>Duvan Camilo</t>
+    <t>$Q5U_CX9_RWX4EVLH</t>
+  </si>
+  <si>
+    <t>ARMANDO REVERÓ</t>
+  </si>
+  <si>
+    <t>14FT%$Ñ%TC8%OWIG</t>
+  </si>
+  <si>
+    <t>Dora Sanatamaría</t>
+  </si>
+  <si>
+    <t>2_Y2LT4_M5G5D_WL0</t>
+  </si>
+  <si>
+    <t>MARIXEL GUEVARA</t>
+  </si>
+  <si>
+    <t>3%NT2%OGPÑ@U&amp;ABT2R</t>
+  </si>
+  <si>
+    <t>Yaqueiry Robinson</t>
+  </si>
+  <si>
+    <t>3RJ2JP6RZOH#KVGIX</t>
+  </si>
+  <si>
+    <t>Nathyavet Oliveros</t>
+  </si>
+  <si>
+    <t>3W4RT32CG4E7UB0BAB</t>
+  </si>
+  <si>
+    <t>Mariley Marlyn Vergara Pérez</t>
+  </si>
+  <si>
+    <t>4$ZWUXLATOÑ42IZB4</t>
+  </si>
+  <si>
+    <t>ARIEL LANUZA QUIROZ</t>
+  </si>
+  <si>
+    <t>563SOG5@KP24D5W$P</t>
+  </si>
+  <si>
+    <t>REBECA MEDINA</t>
+  </si>
+  <si>
+    <t>5RRBT@OPU4BTM5@9S</t>
+  </si>
+  <si>
+    <t>Miguel Charris</t>
+  </si>
+  <si>
+    <t>6$SHLY#AB$XW0P5BFB</t>
+  </si>
+  <si>
+    <t>Isabel Muñoz</t>
+  </si>
+  <si>
+    <t>6F%8UUPQÑ69QHYWTU</t>
+  </si>
+  <si>
+    <t>Kathia Irene Vega Del Cid De Quijano</t>
+  </si>
+  <si>
+    <t>6X_Y6L_79GYV23KMA</t>
+  </si>
+  <si>
+    <t>GABRIELA CARCAC</t>
+  </si>
+  <si>
+    <t>AUDITOR INTERNO EN SISTEMAS INTEGRADOS DE GESTIÓN TRINORMA</t>
+  </si>
+  <si>
+    <t>AUDITOR INTERNO EN SISTEMAS DE GESTIÓNANTISOBORNO ISO 37001:2017</t>
+  </si>
+  <si>
+    <t>6ZPTCAA#4@@DP%&amp;#&amp;3</t>
+  </si>
+  <si>
+    <t>JOSEPH MATEO MEZA</t>
+  </si>
+  <si>
+    <t>7EQAA50IUÑAA5O@J7%</t>
+  </si>
+  <si>
+    <t>EDWIN ANIBAL GUERRA LEZCANO</t>
+  </si>
+  <si>
+    <t>8ES1N9AA&amp;4X8RBP7DK</t>
+  </si>
+  <si>
+    <t>David Mendes</t>
+  </si>
+  <si>
+    <t>AB0ÑUTWMÑ8PATA#11@</t>
+  </si>
+  <si>
+    <t>Ulises Martínez Hernández</t>
+  </si>
+  <si>
+    <t>AGÑQ24FÑ@#VF@XTCH</t>
+  </si>
+  <si>
+    <t>Deyra Naomi Marie Garay Arrocha</t>
+  </si>
+  <si>
+    <t>BI#ABUFN024&amp;Ñ6@HFH</t>
+  </si>
+  <si>
+    <t>Marleny Canto Ramos</t>
+  </si>
+  <si>
+    <t>AUDITOR INTERNO EN SISTEMAS DE GESTIÓN ANTISOBORNO ISO 37001:2017</t>
+  </si>
+  <si>
+    <t>CAA1C0C0@PHQYLCDU0</t>
+  </si>
+  <si>
+    <t>Korina Tenorio</t>
+  </si>
+  <si>
+    <t>CAAUAKKSMVY4OXDVV3</t>
+  </si>
+  <si>
+    <t>Antoinett Tapia</t>
+  </si>
+  <si>
+    <t>D5N$@ÑW_GTLCDTO_V</t>
+  </si>
+  <si>
+    <t>KATHERINE MOJICA</t>
+  </si>
+  <si>
+    <t>DAILQAAT35MDJN@DEU</t>
+  </si>
+  <si>
+    <t>ANTONIO CHANG KRUELL</t>
+  </si>
+  <si>
+    <t>DF6AAD96R4$T8@02LV</t>
+  </si>
+  <si>
+    <t>Fabiana A Velásquez</t>
+  </si>
+  <si>
+    <t>DULUC5OP8H6UJE58B</t>
+  </si>
+  <si>
+    <t>KARINA CASTRO SUNGTAO</t>
+  </si>
+  <si>
+    <t>E%M7II2R$QE5WO$E7</t>
+  </si>
+  <si>
+    <t>HENRY JOHN VARGAS CONTRERAS</t>
+  </si>
+  <si>
+    <t>ERXI0@7EX29D8GS6L</t>
+  </si>
+  <si>
+    <t>Anibal de la Ossa Rodríguez</t>
+  </si>
+  <si>
+    <t>FMQIQT&amp;&amp;Y7E3RI7&amp;%</t>
+  </si>
+  <si>
+    <t>María Gómez Gómez</t>
+  </si>
+  <si>
+    <t>FOOO3W4#UR50S0Y#9</t>
+  </si>
+  <si>
+    <t>Lionel Ariel Vergara Domínguez</t>
+  </si>
+  <si>
+    <t>FYI@HUXAAQ4#J2@_X_</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> BELINDA DE LA CRUZ</t>
+  </si>
+  <si>
+    <t>J44XJ5&amp;6P@PRALWQM</t>
+  </si>
+  <si>
+    <t>Luris Avila</t>
+  </si>
+  <si>
+    <t>J44XJ56P@PRALWQM</t>
+  </si>
+  <si>
+    <t>JB6$2$XGAA73Y4OABKP</t>
+  </si>
+  <si>
+    <t>Leinny Mairelys Sánchez Zambrano</t>
+  </si>
+  <si>
+    <t>KAB5P$XRSC0$3MDN</t>
+  </si>
+  <si>
+    <t>Stephanie Vivero</t>
+  </si>
+  <si>
+    <t>Erika Lizbeth Riquelme Franco</t>
+  </si>
+  <si>
+    <t>L41S2002Y8AAV6GFR</t>
+  </si>
+  <si>
+    <t>LEPEU83KAV5AB7AAR6@</t>
+  </si>
+  <si>
+    <t>Iliana Espinosa</t>
+  </si>
+  <si>
+    <t>LZELC7BQÑ$TAB67@</t>
+  </si>
+  <si>
+    <t>Irma Ocaña</t>
+  </si>
+  <si>
+    <t>MUÑVMDJOB9ZB&amp;HS9T</t>
+  </si>
+  <si>
+    <t>YESIBEL LIZBETH ALDERETE SANTO</t>
+  </si>
+  <si>
+    <t>N10LF3R2YZYQ03Y8</t>
+  </si>
+  <si>
+    <t>Maria De Lourdes Castillero Espino</t>
+  </si>
+  <si>
+    <t>Ñ8TLLP@N&amp;33HKFQWR</t>
+  </si>
+  <si>
+    <t>Kathia Irene Vega Del Cid de Quijano</t>
+  </si>
+  <si>
+    <t>NT4I&amp;AB$BXTTPSDT#D</t>
+  </si>
+  <si>
+    <t>Camila Andrea Quijano Vega</t>
+  </si>
+  <si>
+    <t>ÑTJ0S&amp;ZSHZMSYBXDK</t>
+  </si>
+  <si>
+    <t>Carlos Ariza</t>
+  </si>
+  <si>
+    <t>O%X2WG055XCTH23ÑT</t>
+  </si>
+  <si>
+    <t>Michelle Joanne Nicholson Fernández</t>
+  </si>
+  <si>
+    <t>OAAW2SAA6UFB3FN$19F</t>
+  </si>
+  <si>
+    <t>Virginia Córdoba</t>
+  </si>
+  <si>
+    <t>PNHNDXX4Z%MUR$6JV</t>
+  </si>
+  <si>
+    <t>Ingrid Esther Quezada Castrellón</t>
+  </si>
+  <si>
+    <t>PT$7BAFGICFLRJOM6</t>
+  </si>
+  <si>
+    <t>Amadis Aparicio</t>
+  </si>
+  <si>
+    <t>QB&amp;YOAA25ME2CGIK$@</t>
+  </si>
+  <si>
+    <t>ANGELY ELENA VASQUEZ SANCHEZ</t>
+  </si>
+  <si>
+    <t>QC0ZZFRG97TXKPBCS</t>
+  </si>
+  <si>
+    <t>Angel S. Sánchez</t>
+  </si>
+  <si>
+    <t>QY_HABL332UF9D1HGA</t>
+  </si>
+  <si>
+    <t>ERIC TONG</t>
+  </si>
+  <si>
+    <t>RFIC54B9SB78#J8B9</t>
+  </si>
+  <si>
+    <t>Vanessa Aldazoro J</t>
+  </si>
+  <si>
+    <t>RYÑ4#F#E@AA86826H6</t>
+  </si>
+  <si>
+    <t>MARYORIE MAGDIEL MACKAY ZUÑIGA</t>
+  </si>
+  <si>
+    <t>T$1Q9AAGKRMGAAÑQOL</t>
+  </si>
+  <si>
+    <t>Clarissa Prado</t>
+  </si>
+  <si>
+    <t>T3VWSWL#7SNRP$BQN</t>
+  </si>
+  <si>
+    <t>NIVIELKA J. JEMMOTT V.</t>
+  </si>
+  <si>
+    <t>UO%FÑOZOUK0WAAB92I</t>
+  </si>
+  <si>
+    <t>Estefany Ramos Barrante</t>
+  </si>
+  <si>
+    <t>URABUZ#8WEVEPGE0GB</t>
+  </si>
+  <si>
+    <t>Giovanna Chirú</t>
+  </si>
+  <si>
+    <t>VABPAB6O@1H%1KG5P3</t>
+  </si>
+  <si>
+    <t>Larissa Castillo</t>
+  </si>
+  <si>
+    <t>VÑFUIÑ38MEVMEFG6A</t>
+  </si>
+  <si>
+    <t>JORGE L. GONZÁLEZ A.</t>
+  </si>
+  <si>
+    <t>WQTA$RAAEYOM7JSWSG</t>
+  </si>
+  <si>
+    <t>ANETH BEITIA</t>
+  </si>
+  <si>
+    <t>XARK645TCKH$HKG3B</t>
+  </si>
+  <si>
+    <t>Abdiel Adonis Reyes Goodridge</t>
+  </si>
+  <si>
+    <t>XBSABCL4103A#Y$I%&amp;</t>
+  </si>
+  <si>
+    <t>Alfredo Oliver Graell</t>
+  </si>
+  <si>
+    <t>YCAT0HBRG$YWHAAÑF6</t>
+  </si>
+  <si>
+    <t>Wendie Young</t>
+  </si>
+  <si>
+    <t>ZVIZ#Ñ@D9GRKAAABCAF</t>
+  </si>
+  <si>
+    <t>Alexis A. Rodríguez V.</t>
+  </si>
+  <si>
+    <t>_OAANO1$ABOSK8$VDYÑ</t>
+  </si>
+  <si>
+    <t>FULVIA XIOMARA GARRIDO GÓMEZ</t>
   </si>
 </sst>
 </file>
@@ -112,8 +487,8 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -429,39 +804,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1ED78EBC-390D-4A45-8A90-C0D493A75DE1}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31.85546875" customWidth="1"/>
-    <col min="2" max="2" width="90.140625" customWidth="1"/>
-    <col min="3" max="3" width="29" style="1" customWidth="1"/>
+    <col min="1" max="1" width="26.7109375" customWidth="1"/>
+    <col min="2" max="2" width="31.85546875" customWidth="1"/>
+    <col min="3" max="3" width="108.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="C2" t="s">
         <v>6</v>
       </c>
     </row>
@@ -470,45 +842,691 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="1">
+        <v>45253.621527777781</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>41</v>
+      </c>
+      <c r="B19" t="s">
+        <v>42</v>
+      </c>
+      <c r="C19" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>43</v>
+      </c>
+      <c r="B20" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>46</v>
+      </c>
+      <c r="B21" t="s">
+        <v>47</v>
+      </c>
+      <c r="C21" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>48</v>
+      </c>
+      <c r="B22" t="s">
+        <v>49</v>
+      </c>
+      <c r="C22" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>50</v>
+      </c>
+      <c r="B23" t="s">
+        <v>51</v>
+      </c>
+      <c r="C23" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>52</v>
+      </c>
+      <c r="B24" t="s">
+        <v>53</v>
+      </c>
+      <c r="C24" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>54</v>
+      </c>
+      <c r="B25" t="s">
+        <v>55</v>
+      </c>
+      <c r="C25" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>56</v>
+      </c>
+      <c r="B26" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>58</v>
+      </c>
+      <c r="B27" t="s">
+        <v>59</v>
+      </c>
+      <c r="C27" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>60</v>
+      </c>
+      <c r="B28" t="s">
+        <v>61</v>
+      </c>
+      <c r="C28" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>62</v>
+      </c>
+      <c r="B29" t="s">
+        <v>63</v>
+      </c>
+      <c r="C29" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>64</v>
+      </c>
+      <c r="B30" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>66</v>
+      </c>
+      <c r="B31" t="s">
+        <v>67</v>
+      </c>
+      <c r="C31" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>68</v>
+      </c>
+      <c r="B32" t="s">
+        <v>69</v>
+      </c>
+      <c r="C32" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>70</v>
+      </c>
+      <c r="B33" t="s">
+        <v>69</v>
+      </c>
+      <c r="C33" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>71</v>
+      </c>
+      <c r="B34" t="s">
+        <v>72</v>
+      </c>
+      <c r="C34" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>73</v>
+      </c>
+      <c r="B35" t="s">
+        <v>74</v>
+      </c>
+      <c r="C35" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>76</v>
+      </c>
+      <c r="B36" t="s">
+        <v>75</v>
+      </c>
+      <c r="C36" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B37" t="s">
+        <v>78</v>
+      </c>
+      <c r="C37" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>79</v>
+      </c>
+      <c r="B38" t="s">
+        <v>80</v>
+      </c>
+      <c r="C38" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>81</v>
+      </c>
+      <c r="B39" t="s">
+        <v>82</v>
+      </c>
+      <c r="C39" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>83</v>
+      </c>
+      <c r="B40" t="s">
+        <v>84</v>
+      </c>
+      <c r="C40" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>85</v>
+      </c>
+      <c r="B41" t="s">
+        <v>86</v>
+      </c>
+      <c r="C41" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>87</v>
+      </c>
+      <c r="B42" t="s">
+        <v>88</v>
+      </c>
+      <c r="C42" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>89</v>
+      </c>
+      <c r="B43" t="s">
+        <v>90</v>
+      </c>
+      <c r="C43" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>91</v>
+      </c>
+      <c r="B44" t="s">
+        <v>92</v>
+      </c>
+      <c r="C44" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>93</v>
+      </c>
+      <c r="B45" t="s">
+        <v>94</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>95</v>
+      </c>
+      <c r="B46" t="s">
+        <v>96</v>
+      </c>
+      <c r="C46" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>97</v>
+      </c>
+      <c r="B47" t="s">
+        <v>98</v>
+      </c>
+      <c r="C47" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>99</v>
+      </c>
+      <c r="B48" t="s">
+        <v>100</v>
+      </c>
+      <c r="C48" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>101</v>
+      </c>
+      <c r="B49" t="s">
+        <v>102</v>
+      </c>
+      <c r="C49" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>103</v>
+      </c>
+      <c r="B50" t="s">
+        <v>104</v>
+      </c>
+      <c r="C50" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>105</v>
+      </c>
+      <c r="B51" t="s">
+        <v>106</v>
+      </c>
+      <c r="C51" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>107</v>
+      </c>
+      <c r="B52" t="s">
+        <v>108</v>
+      </c>
+      <c r="C52" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>109</v>
+      </c>
+      <c r="B53" t="s">
+        <v>110</v>
+      </c>
+      <c r="C53" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>111</v>
+      </c>
+      <c r="B54" t="s">
+        <v>112</v>
+      </c>
+      <c r="C54" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>113</v>
+      </c>
+      <c r="B55" t="s">
+        <v>114</v>
+      </c>
+      <c r="C55" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>115</v>
+      </c>
+      <c r="B56" t="s">
+        <v>116</v>
+      </c>
+      <c r="C56" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>117</v>
+      </c>
+      <c r="B57" t="s">
+        <v>118</v>
+      </c>
+      <c r="C57" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>119</v>
+      </c>
+      <c r="B58" t="s">
+        <v>120</v>
+      </c>
+      <c r="C58" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>121</v>
+      </c>
+      <c r="B59" t="s">
+        <v>122</v>
+      </c>
+      <c r="C59" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>123</v>
+      </c>
+      <c r="B60" t="s">
+        <v>124</v>
+      </c>
+      <c r="C60" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>125</v>
+      </c>
+      <c r="B61" t="s">
+        <v>126</v>
+      </c>
+      <c r="C61" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>127</v>
+      </c>
+      <c r="B62" t="s">
+        <v>128</v>
+      </c>
+      <c r="C62" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>129</v>
+      </c>
+      <c r="B63" t="s">
+        <v>130</v>
+      </c>
+      <c r="C63" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>131</v>
+      </c>
+      <c r="B64" t="s">
+        <v>132</v>
+      </c>
+      <c r="C64" t="s">
         <v>6</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{3D3C0B69-1A92-461D-A85D-570BDDB7EEDD}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>